<commit_message>
Updated on SFTP login details SOUTHERNCOMPANYELEC
</commit_message>
<xml_diff>
--- a/EDI_Project_Documentation/FTP-SFTP-Connection Details.xlsx
+++ b/EDI_Project_Documentation/FTP-SFTP-Connection Details.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RPAdmin\Desktop\FInal-SOP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E678E12B-78B8-4919-A3D6-52F9C3871BFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EE225E8-16B5-4C03-B813-750FB55D8666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="139">
   <si>
     <t>No</t>
   </si>
@@ -440,6 +440,9 @@
   </si>
   <si>
     <t>vABCjbXJazbPrHvv</t>
+  </si>
+  <si>
+    <t>vCT4WsR4EACQa6T8</t>
   </si>
 </sst>
 </file>
@@ -2003,7 +2006,7 @@
         <v>68</v>
       </c>
       <c r="F11" s="22" t="s">
-        <v>57</v>
+        <v>138</v>
       </c>
       <c r="G11" s="40" t="s">
         <v>129</v>

</xml_diff>